<commit_message>
Add workspace configuration file for project setup
</commit_message>
<xml_diff>
--- a/Iowa_Distribution_Test_Systems/OpenDSS Model/OpenDSS Model/Rede_240Bus_Dados.xlsx
+++ b/Iowa_Distribution_Test_Systems/OpenDSS Model/OpenDSS Model/Rede_240Bus_Dados.xlsx
@@ -11408,7 +11408,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11429,7 +11429,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11450,7 +11450,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11471,7 +11471,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11492,7 +11492,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11513,7 +11513,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11534,7 +11534,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11555,7 +11555,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11576,7 +11576,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11597,7 +11597,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11618,7 +11618,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11639,7 +11639,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11660,7 +11660,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11681,7 +11681,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11702,7 +11702,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11723,7 +11723,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11744,7 +11744,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11765,7 +11765,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11786,7 +11786,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11807,7 +11807,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11828,7 +11828,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11849,7 +11849,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11870,7 +11870,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11891,7 +11891,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11912,7 +11912,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11933,7 +11933,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11954,7 +11954,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11975,7 +11975,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -11996,7 +11996,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12017,7 +12017,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12038,7 +12038,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12059,7 +12059,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12080,7 +12080,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12227,7 +12227,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12248,7 +12248,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12269,7 +12269,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12290,7 +12290,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12311,7 +12311,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12332,7 +12332,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12353,7 +12353,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12374,7 +12374,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12395,7 +12395,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12416,7 +12416,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12437,7 +12437,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12458,7 +12458,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12479,7 +12479,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12500,7 +12500,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12521,7 +12521,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12542,7 +12542,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12563,7 +12563,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12584,7 +12584,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12605,7 +12605,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12626,7 +12626,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12647,7 +12647,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12668,7 +12668,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12689,7 +12689,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12710,7 +12710,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12731,7 +12731,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12752,7 +12752,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12773,7 +12773,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12794,7 +12794,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12815,7 +12815,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12836,7 +12836,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12857,7 +12857,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12878,7 +12878,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12899,7 +12899,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12920,7 +12920,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12941,7 +12941,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -13025,7 +13025,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -13046,7 +13046,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -13235,7 +13235,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -13256,7 +13256,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -13277,7 +13277,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -13298,7 +13298,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -13319,7 +13319,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -13340,7 +13340,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -13403,7 +13403,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -13424,7 +13424,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -13655,7 +13655,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -13676,7 +13676,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -13949,7 +13949,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -13970,7 +13970,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -13991,7 +13991,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -14012,7 +14012,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -14075,7 +14075,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -14096,7 +14096,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -14201,7 +14201,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -14222,7 +14222,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -14243,7 +14243,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -14264,7 +14264,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -14579,7 +14579,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -14600,7 +14600,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -14915,7 +14915,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -14936,7 +14936,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -14957,7 +14957,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -14978,7 +14978,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -14999,7 +14999,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15020,7 +15020,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15041,7 +15041,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15062,7 +15062,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15083,7 +15083,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15104,7 +15104,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15125,7 +15125,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15146,7 +15146,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15167,7 +15167,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15188,7 +15188,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15209,7 +15209,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15230,7 +15230,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15671,7 +15671,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15692,7 +15692,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15713,7 +15713,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15734,7 +15734,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15797,7 +15797,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15818,7 +15818,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15839,7 +15839,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15860,7 +15860,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15881,7 +15881,7 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15902,7 +15902,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15923,7 +15923,7 @@
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15944,7 +15944,7 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15965,7 +15965,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -15986,7 +15986,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16007,7 +16007,7 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16028,7 +16028,7 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16049,7 +16049,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16070,7 +16070,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16091,7 +16091,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16112,7 +16112,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16133,7 +16133,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16154,7 +16154,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16175,7 +16175,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16196,7 +16196,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16217,7 +16217,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16238,7 +16238,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16259,7 +16259,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16280,7 +16280,7 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16301,7 +16301,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16322,7 +16322,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16343,7 +16343,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16364,7 +16364,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16385,7 +16385,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16406,7 +16406,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16427,7 +16427,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16448,7 +16448,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16469,7 +16469,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16490,7 +16490,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16511,7 +16511,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16532,7 +16532,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16553,7 +16553,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16574,7 +16574,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16763,7 +16763,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16784,7 +16784,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16805,7 +16805,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16826,7 +16826,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16847,7 +16847,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16868,7 +16868,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16889,7 +16889,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16910,7 +16910,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16931,7 +16931,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16952,7 +16952,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16973,7 +16973,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -16994,7 +16994,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17183,7 +17183,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17204,7 +17204,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17309,7 +17309,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17330,7 +17330,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17351,7 +17351,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17372,7 +17372,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17645,7 +17645,7 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17666,7 +17666,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17687,7 +17687,7 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17708,7 +17708,7 @@
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17729,7 +17729,7 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17750,7 +17750,7 @@
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17813,7 +17813,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17834,7 +17834,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17897,7 +17897,7 @@
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17918,7 +17918,7 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17939,7 +17939,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17960,7 +17960,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -17981,7 +17981,7 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18002,7 +18002,7 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18023,7 +18023,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18044,7 +18044,7 @@
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18107,7 +18107,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18128,7 +18128,7 @@
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18149,7 +18149,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18170,7 +18170,7 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18191,7 +18191,7 @@
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18212,7 +18212,7 @@
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18233,7 +18233,7 @@
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18254,7 +18254,7 @@
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18275,7 +18275,7 @@
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18296,7 +18296,7 @@
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18317,7 +18317,7 @@
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18338,7 +18338,7 @@
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18359,7 +18359,7 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18380,7 +18380,7 @@
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18401,7 +18401,7 @@
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18422,7 +18422,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18485,7 +18485,7 @@
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18506,7 +18506,7 @@
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18527,7 +18527,7 @@
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18548,7 +18548,7 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18569,7 +18569,7 @@
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18590,7 +18590,7 @@
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18611,7 +18611,7 @@
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18632,7 +18632,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18653,7 +18653,7 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18674,7 +18674,7 @@
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18695,7 +18695,7 @@
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18716,7 +18716,7 @@
       </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18779,7 +18779,7 @@
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18800,7 +18800,7 @@
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18821,7 +18821,7 @@
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18842,7 +18842,7 @@
       </c>
       <c r="E356" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18863,7 +18863,7 @@
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18884,7 +18884,7 @@
       </c>
       <c r="E358" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18905,7 +18905,7 @@
       </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18926,7 +18926,7 @@
       </c>
       <c r="E360" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18947,7 +18947,7 @@
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18968,7 +18968,7 @@
       </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -18989,7 +18989,7 @@
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19010,7 +19010,7 @@
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19115,7 +19115,7 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19136,7 +19136,7 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19157,7 +19157,7 @@
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19178,7 +19178,7 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19199,7 +19199,7 @@
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19220,7 +19220,7 @@
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19241,7 +19241,7 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19262,7 +19262,7 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19283,7 +19283,7 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19304,7 +19304,7 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19325,7 +19325,7 @@
       </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19346,7 +19346,7 @@
       </c>
       <c r="E380" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19367,7 +19367,7 @@
       </c>
       <c r="E381" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19388,7 +19388,7 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19409,7 +19409,7 @@
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19430,7 +19430,7 @@
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19451,7 +19451,7 @@
       </c>
       <c r="E385" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19472,7 @@
       </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19493,7 +19493,7 @@
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19514,7 +19514,7 @@
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19535,7 +19535,7 @@
       </c>
       <c r="E389" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19556,7 +19556,7 @@
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19577,7 +19577,7 @@
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19598,7 +19598,7 @@
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19619,7 +19619,7 @@
       </c>
       <c r="E393" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19640,7 +19640,7 @@
       </c>
       <c r="E394" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19661,7 +19661,7 @@
       </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19703,7 +19703,7 @@
       </c>
       <c r="E397" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19724,7 +19724,7 @@
       </c>
       <c r="E398" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19745,7 +19745,7 @@
       </c>
       <c r="E399" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       </c>
       <c r="E400" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19787,7 +19787,7 @@
       </c>
       <c r="E401" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19808,7 +19808,7 @@
       </c>
       <c r="E402" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19829,7 +19829,7 @@
       </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19934,7 +19934,7 @@
       </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19955,7 +19955,7 @@
       </c>
       <c r="E409" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -19997,7 +19997,7 @@
       </c>
       <c r="E411" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20018,7 +20018,7 @@
       </c>
       <c r="E412" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20039,7 +20039,7 @@
       </c>
       <c r="E413" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20060,7 +20060,7 @@
       </c>
       <c r="E414" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20081,7 +20081,7 @@
       </c>
       <c r="E415" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20102,7 +20102,7 @@
       </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20123,7 +20123,7 @@
       </c>
       <c r="E417" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20186,7 +20186,7 @@
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20228,7 +20228,7 @@
       </c>
       <c r="E422" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20249,7 +20249,7 @@
       </c>
       <c r="E423" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20270,7 +20270,7 @@
       </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20291,7 +20291,7 @@
       </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20312,7 +20312,7 @@
       </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20333,7 +20333,7 @@
       </c>
       <c r="E427" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20354,7 +20354,7 @@
       </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20375,7 +20375,7 @@
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20396,7 +20396,7 @@
       </c>
       <c r="E430" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -20417,7 +20417,7 @@
       </c>
       <c r="E431" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>

</xml_diff>